<commit_message>
fix: 修复 Luban 生成 DataTableManager 重复冲突，新增 scene/entity 表
- 删除 Gen/DataTableManager.cs（与 Manager/ 下手写版本冲突）
- 修复 gen.bat 不再备份恢复 DataTableManager.cs
- 新增 scene 表和 entity 表（Luban 生成代码 + 数据文件）
</commit_message>
<xml_diff>
--- a/DataTables/Datas/__tables__.xlsx
+++ b/DataTables/Datas/__tables__.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -965,6 +965,86 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>cfg.scene.TbScene</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Scene</t>
+        </is>
+      </c>
+      <c r="D14" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>scene.xlsx</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>场景表</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>cfg.entity.TbEntity</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Entity</t>
+        </is>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>entity.xlsx</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>实体表</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>